<commit_message>
Just solved the ArrayMinMax problem
</commit_message>
<xml_diff>
--- a/FINAL450.xlsx
+++ b/FINAL450.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Me\Shashwat@2026\Job\Private\Goal\Final_450\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7251CEC-8623-400C-94C7-4E8EC11E45D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F24CB82E-02F7-4634-8345-E4183B97076F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{261C335C-1D91-C143-AEEF-19B82073468C}"/>
   </bookViews>
@@ -1894,7 +1894,7 @@
         <v>6</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>4</v>
+        <v>465</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="21">

</xml_diff>